<commit_message>
feature: update new code
</commit_message>
<xml_diff>
--- a/docs/design/ACSMS-SCR-010/【日本農業新聞様】VTIジャパン_クラウド版購読者管理システム_API設計書_メニュー画面_V1.0.xlsx
+++ b/docs/design/ACSMS-SCR-010/【日本農業新聞様】VTIジャパン_クラウド版購読者管理システム_API設計書_メニュー画面_V1.0.xlsx
@@ -1700,7 +1700,7 @@
       <c r="AC2" s="22" t="n"/>
       <c r="AD2" s="23" t="inlineStr">
         <is>
-          <t>2026/04/17</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="AE2" s="21" t="n"/>
@@ -2171,7 +2171,7 @@
       <c r="AC2" s="22" t="n"/>
       <c r="AD2" s="23" t="inlineStr">
         <is>
-          <t>2026/04/17</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="AE2" s="21" t="n"/>
@@ -2815,7 +2815,7 @@
       <c r="AC2" s="22" t="n"/>
       <c r="AD2" s="23" t="inlineStr">
         <is>
-          <t>2026/04/17</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="AE2" s="21" t="n"/>
@@ -3250,7 +3250,7 @@
       <c r="AC2" s="22" t="n"/>
       <c r="AD2" s="23" t="inlineStr">
         <is>
-          <t>2026/04/17</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="AE2" s="21" t="n"/>
@@ -5484,7 +5484,7 @@
     <row r="67" ht="18" customHeight="1">
       <c r="C67" s="41" t="inlineStr">
         <is>
-          <t>認証情報を検証する（JWT / Cookie）。</t>
+          <t>認証情報を検証する（HTTP-only Cookieセッション）。</t>
         </is>
       </c>
     </row>
@@ -6156,7 +6156,7 @@
       <c r="AC2" s="22" t="n"/>
       <c r="AD2" s="23" t="inlineStr">
         <is>
-          <t>2026/04/17</t>
+          <t>2026/04/24</t>
         </is>
       </c>
       <c r="AE2" s="21" t="n"/>
@@ -7381,7 +7381,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="C53" s="41" t="inlineStr">
         <is>
-          <t>認証情報を検証する（JWT / Cookie）。</t>
+          <t>認証情報を検証する（HTTP-only Cookieセッション）。</t>
         </is>
       </c>
     </row>

</xml_diff>